<commit_message>
addition of free convection correlations and their tests in TAeZoSysPro.HeatTransfer.Functions.FreeConvection
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="144525"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>propriétés</t>
   </si>
@@ -96,13 +96,19 @@
     <t>L_...</t>
   </si>
   <si>
-    <t>hcv_...</t>
-  </si>
-  <si>
     <t>Number of node</t>
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>difference Temperature</t>
+  </si>
+  <si>
+    <t>dT</t>
+  </si>
+  <si>
+    <t>h_cv_...</t>
   </si>
 </sst>
 </file>
@@ -444,7 +450,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -452,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
@@ -475,100 +481,108 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="6" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+    <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
addition of the function to determine the radiative heat exchange coefficient + a test of this function in TAeZoSysPro.HeatTransfer.Functions.Radiation
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>propriétés</t>
   </si>
@@ -109,6 +109,18 @@
   </si>
   <si>
     <t>h_cv_...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Radiative heat exchange coefficient </t>
+  </si>
+  <si>
+    <t>h_rad_...</t>
+  </si>
+  <si>
+    <t>emissivity</t>
+  </si>
+  <si>
+    <t>eps_</t>
   </si>
 </sst>
 </file>
@@ -170,13 +182,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -450,7 +468,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -458,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
@@ -546,42 +564,58 @@
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+    <row r="13" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+    <row r="15" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
addition of the convection module and its test in TAeZoSysPro.HeatTransfer.BasesClasses
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -19,13 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
-  <si>
-    <t>propriétés</t>
-  </si>
-  <si>
-    <t>diminutif</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
   <si>
     <t>Temperature</t>
   </si>
@@ -33,81 +27,36 @@
     <t>T_...</t>
   </si>
   <si>
-    <t>Apport de chaleur</t>
-  </si>
-  <si>
     <t>Q_flow_...</t>
   </si>
   <si>
-    <t>Transport de chaleur</t>
-  </si>
-  <si>
     <t>H_flow_...</t>
   </si>
   <si>
     <t>cp_...</t>
   </si>
   <si>
-    <t>Capacité thermique massique</t>
-  </si>
-  <si>
-    <t>Pression</t>
-  </si>
-  <si>
     <t>p_...</t>
   </si>
   <si>
-    <t>Fraction massique</t>
-  </si>
-  <si>
-    <t>X_...</t>
-  </si>
-  <si>
-    <t>masse volumique</t>
-  </si>
-  <si>
     <t>d_...</t>
   </si>
   <si>
-    <t>conductivité</t>
-  </si>
-  <si>
     <t>k_...</t>
   </si>
   <si>
-    <t>Area - Surface</t>
-  </si>
-  <si>
-    <t>A_</t>
-  </si>
-  <si>
-    <t>Longueur caractéristique</t>
-  </si>
-  <si>
     <t xml:space="preserve">Convective heat exchange coefficient </t>
   </si>
   <si>
-    <t>variable d'ajustement</t>
-  </si>
-  <si>
     <t>add_on_...</t>
   </si>
   <si>
-    <t>L_...</t>
-  </si>
-  <si>
     <t>Number of node</t>
   </si>
   <si>
     <t>N</t>
   </si>
   <si>
-    <t>difference Temperature</t>
-  </si>
-  <si>
-    <t>dT</t>
-  </si>
-  <si>
     <t>h_cv_...</t>
   </si>
   <si>
@@ -117,10 +66,82 @@
     <t>h_rad_...</t>
   </si>
   <si>
-    <t>emissivity</t>
-  </si>
-  <si>
-    <t>eps_</t>
+    <t>Flow variables</t>
+  </si>
+  <si>
+    <t>Potential variables</t>
+  </si>
+  <si>
+    <t>diminutive</t>
+  </si>
+  <si>
+    <t>property</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>Temperature difference</t>
+  </si>
+  <si>
+    <t>dT_...</t>
+  </si>
+  <si>
+    <t>Pressure</t>
+  </si>
+  <si>
+    <t>Pressure difference</t>
+  </si>
+  <si>
+    <t>dp_...</t>
+  </si>
+  <si>
+    <t>Geometrical variables</t>
+  </si>
+  <si>
+    <t>Other variables</t>
+  </si>
+  <si>
+    <t>Specific heat capacity at constant pressure</t>
+  </si>
+  <si>
+    <t>Mass fraction</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>density</t>
+  </si>
+  <si>
+    <t>Conductivity</t>
+  </si>
+  <si>
+    <t>Emissivity</t>
+  </si>
+  <si>
+    <t>eps_...</t>
+  </si>
+  <si>
+    <t>(surface) Area</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Characteristic length</t>
+  </si>
+  <si>
+    <t>Lc_...</t>
+  </si>
+  <si>
+    <t>adjusting variable</t>
+  </si>
+  <si>
+    <t>Heat flow (throught tight boundary)</t>
+  </si>
+  <si>
+    <t>Enthalpy flow (transport)</t>
   </si>
 </sst>
 </file>
@@ -136,15 +157,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -171,30 +204,76 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -476,150 +555,321 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B17"/>
+  <dimension ref="B2:O19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.140625" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" customWidth="1"/>
+    <col min="9" max="9" width="18.42578125" customWidth="1"/>
+    <col min="13" max="13" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="13"/>
+      <c r="E2" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="I2" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="M2" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="N2" s="15"/>
+      <c r="O2" s="15"/>
+    </row>
+    <row r="3" spans="2:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="G4" s="1"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" s="1"/>
+      <c r="M4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="N4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="O4" s="1"/>
+    </row>
+    <row r="5" spans="2:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="E5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="1"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K5" s="1"/>
+      <c r="M5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="1"/>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="E6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6" s="1"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="M6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="2:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="E7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="1"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="M7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O7" s="1"/>
+    </row>
+    <row r="8" spans="2:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="E8" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="F8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="1"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="M8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="O8" s="1"/>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="E9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="G9" s="1"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="M9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="O9" s="1"/>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B10" s="9"/>
+      <c r="C10" s="10"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="M10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="N10" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="O10" s="1"/>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="5"/>
+      <c r="O11" s="5"/>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="M2:O2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
addition of the conduction module and its test in TAeZoSysPro.HeatTransfer.BasesClasses + mistakes fix in HTML description of other modules
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
   <si>
     <t>Temperature</t>
   </si>
@@ -142,6 +142,18 @@
   </si>
   <si>
     <t>Enthalpy flow (transport)</t>
+  </si>
+  <si>
+    <t>Length</t>
+  </si>
+  <si>
+    <t>L _...</t>
+  </si>
+  <si>
+    <t>Thickness</t>
+  </si>
+  <si>
+    <t>Th</t>
   </si>
 </sst>
 </file>
@@ -547,7 +559,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -688,9 +700,13 @@
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
+      <c r="I6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="K6" s="1"/>
       <c r="M6" s="1" t="s">
         <v>32</v>
       </c>
@@ -710,9 +726,13 @@
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
+      <c r="I7" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K7" s="1"/>
       <c r="M7" s="2" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
change the h_rad function to have as input the thermal resistance rather than only the emissivity
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="47">
   <si>
     <t>Temperature</t>
   </si>
@@ -154,6 +154,12 @@
   </si>
   <si>
     <t>Th</t>
+  </si>
+  <si>
+    <t>Thermal resistance</t>
+  </si>
+  <si>
+    <t>R_th_...</t>
   </si>
 </sst>
 </file>
@@ -559,7 +565,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -776,10 +782,10 @@
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
       <c r="M9" s="2" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="O9" s="1"/>
     </row>
@@ -792,12 +798,8 @@
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
-      <c r="M10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
       <c r="O10" s="1"/>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
@@ -809,9 +811,13 @@
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
+      <c r="M11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="O11" s="1"/>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B12" s="9"/>
@@ -822,9 +828,13 @@
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
+      <c r="M12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O12" s="1"/>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B13" s="9"/>

</xml_diff>

<commit_message>
Addition of the PartialWall module and its test in TAeZoSysPro.HeatTransfer.BasesClasses
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="49">
   <si>
     <t>Temperature</t>
   </si>
@@ -160,6 +160,12 @@
   </si>
   <si>
     <t>R_th_...</t>
+  </si>
+  <si>
+    <t>Thermal diffusivity</t>
+  </si>
+  <si>
+    <t>D_th_...</t>
   </si>
 </sst>
 </file>
@@ -565,7 +571,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -721,7 +727,7 @@
       </c>
       <c r="O6" s="1"/>
     </row>
-    <row r="7" spans="2:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="E7" s="1" t="s">
@@ -739,11 +745,11 @@
         <v>44</v>
       </c>
       <c r="K7" s="1"/>
-      <c r="M7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>12</v>
+      <c r="M7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="O7" s="1"/>
     </row>
@@ -761,14 +767,14 @@
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
       <c r="M8" s="2" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O8" s="1"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:15" ht="45" x14ac:dyDescent="0.25">
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="E9" s="1" t="s">
@@ -782,10 +788,10 @@
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
       <c r="M9" s="2" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="O9" s="1"/>
     </row>
@@ -798,8 +804,12 @@
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
+      <c r="M10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="O10" s="1"/>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
@@ -811,12 +821,8 @@
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
-      <c r="M11" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
       <c r="O11" s="1"/>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
@@ -829,10 +835,10 @@
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
       <c r="M12" s="2" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O12" s="1"/>
     </row>
@@ -845,9 +851,13 @@
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
+      <c r="M13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O13" s="1"/>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B14" s="9"/>

</xml_diff>

<commit_message>
Change the variable name for mass from Mass to m
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="51">
   <si>
     <t>Temperature</t>
   </si>
@@ -108,9 +108,6 @@
     <t>Mass fraction</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
     <t>density</t>
   </si>
   <si>
@@ -126,9 +123,6 @@
     <t>(surface) Area</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
     <t>Characteristic length</t>
   </si>
   <si>
@@ -153,9 +147,6 @@
     <t>Thickness</t>
   </si>
   <si>
-    <t>Th</t>
-  </si>
-  <si>
     <t>Thermal resistance</t>
   </si>
   <si>
@@ -166,6 +157,21 @@
   </si>
   <si>
     <t>D_th_...</t>
+  </si>
+  <si>
+    <t>Th_...</t>
+  </si>
+  <si>
+    <t>X_...</t>
+  </si>
+  <si>
+    <t>A_...</t>
+  </si>
+  <si>
+    <t>Mass</t>
+  </si>
+  <si>
+    <t>m_...</t>
   </si>
 </sst>
 </file>
@@ -571,7 +577,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -612,7 +618,7 @@
     </row>
     <row r="3" spans="2:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>2</v>
@@ -647,7 +653,7 @@
     </row>
     <row r="4" spans="2:15" ht="45" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
@@ -661,10 +667,10 @@
       <c r="G4" s="1"/>
       <c r="H4" s="6"/>
       <c r="I4" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="K4" s="1"/>
       <c r="M4" s="1" t="s">
@@ -687,14 +693,14 @@
       <c r="G5" s="1"/>
       <c r="H5" s="6"/>
       <c r="I5" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K5" s="1"/>
       <c r="M5" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>7</v>
@@ -713,17 +719,17 @@
       <c r="G6" s="1"/>
       <c r="H6" s="6"/>
       <c r="I6" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="K6" s="1"/>
       <c r="M6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N6" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="O6" s="1"/>
     </row>
@@ -739,17 +745,17 @@
       <c r="G7" s="1"/>
       <c r="H7" s="6"/>
       <c r="I7" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K7" s="1"/>
       <c r="M7" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="O7" s="1"/>
     </row>
@@ -760,7 +766,7 @@
         <v>28</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="G8" s="1"/>
       <c r="I8" s="5"/>
@@ -778,7 +784,7 @@
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="E9" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>6</v>
@@ -805,10 +811,10 @@
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
       <c r="M10" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="O10" s="1"/>
     </row>
@@ -835,7 +841,7 @@
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
       <c r="M12" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="N12" s="2" t="s">
         <v>9</v>
@@ -868,9 +874,13 @@
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
+      <c r="M14" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="O14" s="1"/>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B15" s="9"/>

</xml_diff>

<commit_message>
Addition of the LumpVolume and CarrollNode modules and the test of the LumpVolume in TAeZoSysPro.HeatTransfer.BasesClasses
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="53">
   <si>
     <t>Temperature</t>
   </si>
@@ -172,6 +172,12 @@
   </si>
   <si>
     <t>m_...</t>
+  </si>
+  <si>
+    <t>Volume</t>
+  </si>
+  <si>
+    <t>V_...</t>
   </si>
 </sst>
 </file>
@@ -577,7 +583,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -769,9 +775,13 @@
         <v>47</v>
       </c>
       <c r="G8" s="1"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
+      <c r="I8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="K8" s="1"/>
       <c r="M8" s="2" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Addition of the PartialHeatExchanger module in TAeZoSysPro.HeatTransfer.BasesClasses
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="58">
   <si>
     <t>Temperature</t>
   </si>
@@ -178,14 +178,50 @@
   </si>
   <si>
     <t>V_...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heat exchange coefficient </t>
+  </si>
+  <si>
+    <t>h_...</t>
+  </si>
+  <si>
+    <t>Qc_...</t>
+  </si>
+  <si>
+    <t>Thermal flow rate</t>
+  </si>
+  <si>
+    <r>
+      <t>W.K</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-1</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <vertAlign val="superscript"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -266,7 +302,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -310,6 +346,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -583,7 +622,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -811,7 +850,7 @@
       </c>
       <c r="O9" s="1"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B10" s="9"/>
       <c r="C10" s="10"/>
       <c r="E10" s="5"/>
@@ -821,10 +860,10 @@
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
       <c r="M10" s="2" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="O10" s="1"/>
     </row>
@@ -837,8 +876,12 @@
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
+      <c r="M11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="O11" s="1"/>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
@@ -892,12 +935,21 @@
       </c>
       <c r="O14" s="1"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
+      <c r="M15" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="O15" s="16" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B16" s="9"/>
@@ -931,5 +983,6 @@
     <mergeCell ref="M2:O2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Addition of the HeatExchanger module in HeatTransfer.Components + addition of counterCurrent function in HeatTransfer.Functions.ExchangerEffectiveness + addition of the NTU_counterCurrent function that is used as the inverse of the counterCurrent
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="60">
   <si>
     <t>Temperature</t>
   </si>
@@ -206,6 +206,12 @@
       </rPr>
       <t>-1</t>
     </r>
+  </si>
+  <si>
+    <t>Effectiveness</t>
+  </si>
+  <si>
+    <t>Eff_...</t>
   </si>
 </sst>
 </file>
@@ -302,7 +308,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -335,6 +341,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -347,9 +356,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -622,7 +629,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -641,25 +648,25 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="E2" s="14" t="s">
+      <c r="C2" s="14"/>
+      <c r="E2" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="M2" s="15" t="s">
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="M2" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="N2" s="15"/>
-      <c r="O2" s="15"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
     </row>
     <row r="3" spans="2:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
@@ -947,7 +954,7 @@
       <c r="N15" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="O15" s="16" t="s">
+      <c r="O15" s="12" t="s">
         <v>57</v>
       </c>
     </row>
@@ -957,6 +964,13 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
+      <c r="M16" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="O16" s="17"/>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="11"/>

</xml_diff>

<commit_message>
Addition of the Ventilation module in HeatTransfer.Components
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="62">
   <si>
     <t>Temperature</t>
   </si>
@@ -212,6 +212,12 @@
   </si>
   <si>
     <t>Eff_...</t>
+  </si>
+  <si>
+    <t>V_flow_...</t>
+  </si>
+  <si>
+    <t>Volume flow</t>
   </si>
 </sst>
 </file>
@@ -344,6 +350,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -356,7 +363,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -629,7 +635,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -648,25 +654,25 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="E2" s="15" t="s">
+      <c r="C2" s="15"/>
+      <c r="E2" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="I2" s="16" t="s">
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="I2" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="M2" s="16" t="s">
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="M2" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
     </row>
     <row r="3" spans="2:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
@@ -734,8 +740,12 @@
       <c r="O4" s="1"/>
     </row>
     <row r="5" spans="2:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
+      <c r="B5" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="E5" s="1" t="s">
         <v>20</v>
       </c>
@@ -970,7 +980,7 @@
       <c r="N16" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="O16" s="17"/>
+      <c r="O16" s="13"/>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="11"/>

</xml_diff>

<commit_message>
Addition of the FreeConvection module in the FluidDynamics.BasesClasses package
</commit_message>
<xml_diff>
--- a/Normenclature_variables_names.xlsx
+++ b/Normenclature_variables_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="64">
   <si>
     <t>Temperature</t>
   </si>
@@ -218,6 +218,12 @@
   </si>
   <si>
     <t>Volume flow</t>
+  </si>
+  <si>
+    <t>relative humidity</t>
+  </si>
+  <si>
+    <t>RH_...</t>
   </si>
 </sst>
 </file>
@@ -635,7 +641,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -870,9 +876,13 @@
     <row r="10" spans="2:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B10" s="9"/>
       <c r="C10" s="10"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
+      <c r="E10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10" s="1"/>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>

</xml_diff>